<commit_message>
Fix: titre dupliqué entre deux CodeSystem (copier-coller) (#331)
Le CodeSystem fr-core-cs-method-collection avait le même Title
que fr-core-cs-mode-validation-identity, provoquant l'erreur
publisher "multiple resources with the same title" (doublon TOC). 8559a54cd67769299a08a35f3f6d3d20bd0ff6b3
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-fr-core-cs-method-collection.xlsx
+++ b/main/ig/CodeSystem-fr-core-cs-method-collection.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>FR Core CodeSystem Mode Validation Identite</t>
+    <t>FR Core CodeSystem Method Collection</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-03T12:52:25+00:00</t>
+    <t>2026-08-04T12:22:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>